<commit_message>
Stage 2: catalog-motor comparison; battery series count from max voltage
- New date/motoare_catalog.json (YASA, Turntide, Helix, EMRAX,
  Equipmake datasheets) and an auto-generated comparison: 1 x YASA YM360
  + 2 x YM720 meets peak power, continuous power and wheel torque
- Battery: Ns = floor(850 V / 4.2 V) = 202 so the fully charged pack
  stays within 800-850 V motor/inverter ratings (727 V nominal,
  505-848 V); vehicle mean becomes 202s29p, 44 A per cell at U_min
- README: catalog conclusions, inverter voltages and sources updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dz8sSyt3zaur1x4jsnU1sR
</commit_message>
<xml_diff>
--- a/etapa2-calcule/CCA_Etapa2_Calcule.xlsx
+++ b/etapa2-calcule/CCA_Etapa2_Calcule.xlsx
@@ -37,7 +37,7 @@
     <definedName function="false" hidden="false" name="c_r" vbProcedure="false">Ipoteze!$C$11</definedName>
     <definedName function="false" hidden="false" name="c_rez" vbProcedure="false">Ipoteze!$C$17</definedName>
     <definedName function="false" hidden="false" name="c_rho" vbProcedure="false">Ipoteze!$C$6</definedName>
-    <definedName function="false" hidden="false" name="c_U_tinta" vbProcedure="false">Ipoteze!$C$18</definedName>
+    <definedName function="false" hidden="false" name="c_U_max" vbProcedure="false">Ipoteze!$C$18</definedName>
     <definedName function="false" hidden="false" name="c_V1_kmh" vbProcedure="false">Ipoteze!$C$15</definedName>
     <definedName function="false" hidden="false" name="c_Va_kmh" vbProcedure="false">Ipoteze!$C$13</definedName>
     <definedName function="false" hidden="false" name="c_Vv" vbProcedure="false">Ipoteze!$C$10</definedName>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="544">
   <si>
     <t xml:space="preserve">Date din documentare (etapa 1) transformate în unități S.I.</t>
   </si>
@@ -456,13 +456,13 @@
     <t xml:space="preserve">Curs, P3 slide 8</t>
   </si>
   <si>
-    <t xml:space="preserve">c_U_tinta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tensiunea nominală țintă a bateriei</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arhitectura de 800 V a clasei</t>
+    <t xml:space="preserve">c_U_max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tensiunea maximă admisă a bateriei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clasa „800 V”: invertoare / motoare de cel mult 800–850 V (YASA 800 V, EMRAX 830 V, Turntide 850 V)</t>
   </si>
   <si>
     <t xml:space="preserve">c_k_masa</t>
@@ -1320,7 +1320,7 @@
     <t xml:space="preserve">Ns</t>
   </si>
   <si>
-    <t xml:space="preserve">U_bat ≈ 800 V</t>
+    <t xml:space="preserve">Ns·U_max celulă ≤ tensiunea maximă admisă</t>
   </si>
   <si>
     <t xml:space="preserve">Tensiunea nominală a bateriei</t>
@@ -1624,6 +1624,51 @@
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.3390/wevj11040077</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motoare YASA YM720 / YM360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YASA – Series motors (pagina producătorului)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://yasa.com/yasa-series-motors/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor Turntide AF300D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turntide – Axial flux motors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://turntide.com/products/motors/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor Helix SPM177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Helix – SPM177 electric motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ehelix.com/products/spm177-electric-motor/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor EMRAX 348</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMRAX – fișă tehnică v1.7 (PDF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://emrax.com/wp-content/uploads/2026/08/EMRAX_348_datasheet_v1.7.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor Equipmake APM-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipmake – APM-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://equipmake.com/products/apm-200/</t>
   </si>
   <si>
     <t xml:space="preserve">Metoda de calcul</t>
@@ -3717,11 +3762,11 @@
       </c>
       <c r="D17" s="24" t="str">
         <f aca="false">TEXT(Baterie!E12,"0")&amp;"s × "&amp;TEXT(Baterie!E21,"0")&amp;"p = "&amp;TEXT(Baterie!E22,"0")</f>
-        <v>222s × 27p = 5994</v>
+        <v>202s × 29p = 5858</v>
       </c>
       <c r="E17" s="24" t="str">
         <f aca="false">TEXT(Baterie!F12,"0")&amp;"s × "&amp;TEXT(Baterie!F21,"0")&amp;"p = "&amp;TEXT(Baterie!F22,"0")</f>
-        <v>222s × 31p = 6882</v>
+        <v>202s × 34p = 6868</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3734,11 +3779,11 @@
       </c>
       <c r="D18" s="29" t="n">
         <f aca="false">Baterie!E23</f>
-        <v>107.892</v>
+        <v>105.444</v>
       </c>
       <c r="E18" s="29" t="n">
         <f aca="false">Baterie!F23</f>
-        <v>123.876</v>
+        <v>123.624</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3751,11 +3796,11 @@
       </c>
       <c r="D19" s="24" t="str">
         <f aca="false">TEXT(Baterie!E13,"0")&amp;" ("&amp;TEXT(Baterie!E15,"0")&amp;" – "&amp;TEXT(Baterie!E14,"0")&amp;")"</f>
-        <v>799 (555 – 932)</v>
+        <v>727 (505 – 848)</v>
       </c>
       <c r="E19" s="24" t="str">
         <f aca="false">TEXT(Baterie!F13,"0")&amp;" ("&amp;TEXT(Baterie!F15,"0")&amp;" – "&amp;TEXT(Baterie!F14,"0")&amp;")"</f>
-        <v>799 (555 – 932)</v>
+        <v>727 (505 – 848)</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3768,11 +3813,11 @@
       </c>
       <c r="D20" s="24" t="str">
         <f aca="false">TEXT(Baterie!E31,"0")&amp;" / "&amp;TEXT(Baterie!E32,"0")</f>
-        <v>426 / 676</v>
+        <v>416 / 660</v>
       </c>
       <c r="E20" s="24" t="str">
         <f aca="false">TEXT(Baterie!F31,"0")&amp;" / "&amp;TEXT(Baterie!F32,"0")</f>
-        <v>489 / 776</v>
+        <v>488 / 774</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3804,11 +3849,11 @@
       </c>
       <c r="D22" s="24" t="str">
         <f aca="false">TEXT(Baterie!E18,"0")&amp;" / "&amp;TEXT(Baterie!E19,"0")</f>
-        <v>811 / 1168</v>
+        <v>892 / 1284</v>
       </c>
       <c r="E22" s="24" t="str">
         <f aca="false">TEXT(Baterie!F18,"0")&amp;" / "&amp;TEXT(Baterie!F19,"0")</f>
-        <v>847 / 1220</v>
+        <v>931 / 1341</v>
       </c>
     </row>
   </sheetData>
@@ -4093,7 +4138,7 @@
         <v>135</v>
       </c>
       <c r="C18" s="30" t="n">
-        <v>800</v>
+        <v>850</v>
       </c>
       <c r="D18" s="23" t="s">
         <v>78</v>
@@ -51242,12 +51287,12 @@
         <v>54</v>
       </c>
       <c r="E12" s="38" t="n">
-        <f aca="false">ROUND(c_U_tinta/cel_U_nom,0)</f>
-        <v>222</v>
+        <f aca="false">ROUNDDOWN(c_U_max/cel_U_max,0)</f>
+        <v>202</v>
       </c>
       <c r="F12" s="38" t="n">
-        <f aca="false">ROUND(c_U_tinta/cel_U_nom,0)</f>
-        <v>222</v>
+        <f aca="false">ROUNDDOWN(c_U_max/cel_U_max,0)</f>
+        <v>202</v>
       </c>
       <c r="G12" s="33" t="s">
         <v>422</v>
@@ -51266,11 +51311,11 @@
       </c>
       <c r="E13" s="32" t="n">
         <f aca="false">E12*cel_U_nom</f>
-        <v>799.2</v>
+        <v>727.2</v>
       </c>
       <c r="F13" s="32" t="n">
         <f aca="false">F12*cel_U_nom</f>
-        <v>799.2</v>
+        <v>727.2</v>
       </c>
       <c r="G13" s="33"/>
     </row>
@@ -51285,11 +51330,11 @@
       </c>
       <c r="E14" s="32" t="n">
         <f aca="false">E12*cel_U_max</f>
-        <v>932.4</v>
+        <v>848.4</v>
       </c>
       <c r="F14" s="32" t="n">
         <f aca="false">F12*cel_U_max</f>
-        <v>932.4</v>
+        <v>848.4</v>
       </c>
       <c r="G14" s="33"/>
     </row>
@@ -51304,11 +51349,11 @@
       </c>
       <c r="E15" s="32" t="n">
         <f aca="false">E12*cel_U_min</f>
-        <v>555</v>
+        <v>505</v>
       </c>
       <c r="F15" s="32" t="n">
         <f aca="false">F12*cel_U_min</f>
-        <v>555</v>
+        <v>505</v>
       </c>
       <c r="G15" s="33"/>
     </row>
@@ -51325,11 +51370,11 @@
       </c>
       <c r="E16" s="35" t="n">
         <f aca="false">ROUNDUP(E11/E12,0)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F16" s="35" t="n">
         <f aca="false">ROUNDUP(F11/F12,0)</f>
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G16" s="33"/>
     </row>
@@ -51367,11 +51412,11 @@
       </c>
       <c r="E18" s="32" t="n">
         <f aca="false">E17/E13</f>
-        <v>811.361234972346</v>
+        <v>891.694030514163</v>
       </c>
       <c r="F18" s="32" t="n">
         <f aca="false">F17/F13</f>
-        <v>847.248763915431</v>
+        <v>931.134780144681</v>
       </c>
       <c r="G18" s="33"/>
     </row>
@@ -51388,11 +51433,11 @@
       </c>
       <c r="E19" s="40" t="n">
         <f aca="false">E17/E15</f>
-        <v>1168.36017836018</v>
+        <v>1284.03940394039</v>
       </c>
       <c r="F19" s="40" t="n">
         <f aca="false">F17/F15</f>
-        <v>1220.03822003822</v>
+        <v>1340.83408340834</v>
       </c>
       <c r="G19" s="33" t="s">
         <v>435</v>
@@ -51411,11 +51456,11 @@
       </c>
       <c r="E20" s="35" t="n">
         <f aca="false">ROUNDUP(E19/cel_I,0)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F20" s="35" t="n">
         <f aca="false">ROUNDUP(F19/cel_I,0)</f>
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G20" s="33"/>
     </row>
@@ -51432,11 +51477,11 @@
       </c>
       <c r="E21" s="38" t="n">
         <f aca="false">MAX(E16,E20)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F21" s="38" t="n">
         <f aca="false">MAX(F16,F20)</f>
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G21" s="33"/>
     </row>
@@ -51453,11 +51498,11 @@
       </c>
       <c r="E22" s="38" t="n">
         <f aca="false">E12*E21</f>
-        <v>5994</v>
+        <v>5858</v>
       </c>
       <c r="F22" s="38" t="n">
         <f aca="false">F12*F21</f>
-        <v>6882</v>
+        <v>6868</v>
       </c>
       <c r="G22" s="33"/>
     </row>
@@ -51472,11 +51517,11 @@
       </c>
       <c r="E23" s="41" t="n">
         <f aca="false">E22*E10/3600000</f>
-        <v>107.892</v>
+        <v>105.444</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">F22*F10/3600000</f>
-        <v>123.876</v>
+        <v>123.624</v>
       </c>
       <c r="G23" s="33"/>
     </row>
@@ -51491,11 +51536,11 @@
       </c>
       <c r="E24" s="32" t="n">
         <f aca="false">E21*cel_Cap</f>
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="F24" s="32" t="n">
         <f aca="false">F21*cel_Cap</f>
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="G24" s="33"/>
     </row>
@@ -51510,11 +51555,11 @@
       </c>
       <c r="E25" s="14" t="n">
         <f aca="false">E19/E21</f>
-        <v>43.2725991985251</v>
+        <v>44.2772208255308</v>
       </c>
       <c r="F25" s="14" t="n">
         <f aca="false">F19/F21</f>
-        <v>39.3560716141361</v>
+        <v>39.4362965708336</v>
       </c>
       <c r="G25" s="33" t="s">
         <v>441</v>
@@ -51531,11 +51576,11 @@
       </c>
       <c r="E26" s="14" t="n">
         <f aca="false">E18/E21</f>
-        <v>30.0504161100869</v>
+        <v>30.7480700177297</v>
       </c>
       <c r="F26" s="14" t="n">
         <f aca="false">F18/F21</f>
-        <v>27.3306052875945</v>
+        <v>27.3863170630789</v>
       </c>
       <c r="G26" s="33"/>
     </row>
@@ -51573,11 +51618,11 @@
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">E27/c_eta/E13/E21</f>
-        <v>50.4497553108664</v>
+        <v>51.6210026175031</v>
       </c>
       <c r="F28" s="14" t="n">
         <f aca="false">F27/c_eta/F13/F21</f>
-        <v>43.3901643579063</v>
+        <v>43.4786125671391</v>
       </c>
       <c r="G28" s="33"/>
     </row>
@@ -51592,11 +51637,11 @@
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">E27/c_eta/E15/E21</f>
-        <v>72.6476476476476</v>
+        <v>74.3342437692045</v>
       </c>
       <c r="F29" s="14" t="n">
         <f aca="false">F27/c_eta/F15/F21</f>
-        <v>62.4818366753851</v>
+        <v>62.6092020966803</v>
       </c>
       <c r="G29" s="33" t="s">
         <v>446</v>
@@ -51618,11 +51663,11 @@
       </c>
       <c r="E31" s="40" t="n">
         <f aca="false">E22*cel_m</f>
-        <v>425.574</v>
+        <v>415.918</v>
       </c>
       <c r="F31" s="40" t="n">
         <f aca="false">F22*cel_m</f>
-        <v>488.622</v>
+        <v>487.628</v>
       </c>
       <c r="G31" s="33"/>
     </row>
@@ -51637,11 +51682,11 @@
       </c>
       <c r="E32" s="32" t="n">
         <f aca="false">E31/cel_kcp</f>
-        <v>675.514285714286</v>
+        <v>660.187301587302</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">F31/cel_kcp</f>
-        <v>775.590476190476</v>
+        <v>774.012698412698</v>
       </c>
       <c r="G32" s="33" t="s">
         <v>450</v>
@@ -51677,11 +51722,11 @@
       </c>
       <c r="E34" s="32" t="n">
         <f aca="false">E31/E8*100</f>
-        <v>18.0649460905</v>
+        <v>17.655064097122</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">F31/F8*100</f>
-        <v>19.8626829268293</v>
+        <v>19.8222764227642</v>
       </c>
       <c r="G34" s="33"/>
     </row>
@@ -51696,11 +51741,11 @@
       </c>
       <c r="E35" s="32" t="n">
         <f aca="false">E32/E8*100</f>
-        <v>28.6745176039683</v>
+        <v>28.023911265273</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">F32/F8*100</f>
-        <v>31.5280681378242</v>
+        <v>31.4639308297845</v>
       </c>
       <c r="G35" s="33"/>
     </row>
@@ -51737,7 +51782,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -52010,7 +52055,7 @@
       <c r="B27" s="23" t="s">
         <v>525</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="51" t="s">
         <v>526</v>
       </c>
     </row>
@@ -52021,8 +52066,63 @@
       <c r="B28" s="23" t="s">
         <v>528</v>
       </c>
-      <c r="C28" s="23" t="s">
-        <v>526</v>
+      <c r="C28" s="51" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="23" t="s">
+        <v>530</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>531</v>
+      </c>
+      <c r="C29" s="51" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="23" t="s">
+        <v>533</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>534</v>
+      </c>
+      <c r="C30" s="51" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="23" t="s">
+        <v>536</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>537</v>
+      </c>
+      <c r="C31" s="51" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
+        <v>539</v>
+      </c>
+      <c r="B32" s="23" t="s">
+        <v>540</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="23" t="s">
+        <v>542</v>
+      </c>
+      <c r="B33" s="23" t="s">
+        <v>543</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>541</v>
       </c>
     </row>
   </sheetData>
@@ -52048,6 +52148,11 @@
     <hyperlink ref="C24" r:id="rId19" display="https://www.fueleconomy.gov/feg/atv-ev.shtml"/>
     <hyperlink ref="C25" r:id="rId20" display="https://doi.org/10.3390/wevj16090484"/>
     <hyperlink ref="C26" r:id="rId21" display="https://doi.org/10.3390/wevj11040077"/>
+    <hyperlink ref="C27" r:id="rId22" display="https://yasa.com/yasa-series-motors/"/>
+    <hyperlink ref="C28" r:id="rId23" display="https://turntide.com/products/motors/"/>
+    <hyperlink ref="C29" r:id="rId24" display="https://www.ehelix.com/products/spm177-electric-motor/"/>
+    <hyperlink ref="C30" r:id="rId25" display="https://emrax.com/wp-content/uploads/2026/08/EMRAX_348_datasheet_v1.7.pdf"/>
+    <hyperlink ref="C31" r:id="rId26" display="https://equipmake.com/products/apm-200/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Stage 2: per-axle motor check, 800 V battery limit, final review fixes
- Catalog comparison now checks wheel torque per axle (static 50/50,
  load transfer with h/L = 0.17): 3 x YASA YM720 (1 front + 2 rear)
  meets every requirement; 1 x YM360 + 2 x YM720 fails at the front
- Battery max voltage = lowest component rating (YASA 400-800 V):
  190s31p, 684 V nominal (475-798 V), 44 A per cell at U_min
- README: torque no longer used as a coherence check (depends on n_max),
  rho derivation, Um limited to the linear modulation range, explicit
  note on the discretisation index reading; Excel note fixed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dz8sSyt3zaur1x4jsnU1sR
</commit_message>
<xml_diff>
--- a/etapa2-calcule/CCA_Etapa2_Calcule.xlsx
+++ b/etapa2-calcule/CCA_Etapa2_Calcule.xlsx
@@ -462,7 +462,7 @@
     <t xml:space="preserve">Tensiunea maximă admisă a bateriei</t>
   </si>
   <si>
-    <t xml:space="preserve">Clasa „800 V”: invertoare / motoare de cel mult 800–850 V (YASA 800 V, EMRAX 830 V, Turntide 850 V)</t>
+    <t xml:space="preserve">Minimul tensiunilor admise de componente: motoarele YASA alese sunt date pentru 400–800 V</t>
   </si>
   <si>
     <t xml:space="preserve">c_k_masa</t>
@@ -939,7 +939,7 @@
     <t xml:space="preserve">Accelerația din sesiunea precedentă (P2: a = Va/ta)</t>
   </si>
   <si>
-    <t xml:space="preserve">sesiunea precedentă (P2, pasul 4)</t>
+    <t xml:space="preserve">sesiunea precedentă (P2, pasul 2: a = Va/ta); aderența se verifică la V1 (pasul 4)</t>
   </si>
   <si>
     <t xml:space="preserve">Pașii 1–6: puterea P1 (cu a), P1' (fără a), timpul t1</t>
@@ -1248,7 +1248,7 @@
     <t xml:space="preserve">P3 – discretizarea intervalului [0, t1] în n = 100 intervale egale</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicii ca în curs (și în Matlab): i = 1 … n+1, t_i = (i − 1)·Δt. P01-med = (1/n)·Σ(i=1..n) Fti·Vti folosește valorile de la începutul intervalelor; W01 = Σ(i=1..n+1) Pti·Δt, cu P(t_1) = 0, folosește valorile de la sfârșitul intervalelor. Cele două sume încadrează valoarea exactă.</t>
+    <t xml:space="preserve">Indicii ca în curs (și în Matlab): i = 1 … n+1, t_i = (i − 1)·Δt. P01-med = (1/n)·Σ(i=1..n) Fti·Vti folosește valorile de la începutul intervalelor; W01 = Σ(i=1..n+1) Pti·Δt, cu P(t_1) = 0, folosește valorile de la sfârșitul intervalelor. Cele două sume încadrează valoarea exactă. (Notația [Δt(i−1), Δt(i)] de pe slide-ul 5 ar asocia Fti sfârșitului intervalului; s-a păstrat forma sumelor din curs.)</t>
   </si>
   <si>
     <t xml:space="preserve">GT 63</t>
@@ -3762,11 +3762,11 @@
       </c>
       <c r="D17" s="24" t="str">
         <f aca="false">TEXT(Baterie!E12,"0")&amp;"s × "&amp;TEXT(Baterie!E21,"0")&amp;"p = "&amp;TEXT(Baterie!E22,"0")</f>
-        <v>202s × 29p = 5858</v>
+        <v>190s × 31p = 5890</v>
       </c>
       <c r="E17" s="24" t="str">
         <f aca="false">TEXT(Baterie!F12,"0")&amp;"s × "&amp;TEXT(Baterie!F21,"0")&amp;"p = "&amp;TEXT(Baterie!F22,"0")</f>
-        <v>202s × 34p = 6868</v>
+        <v>190s × 36p = 6840</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3779,11 +3779,11 @@
       </c>
       <c r="D18" s="29" t="n">
         <f aca="false">Baterie!E23</f>
-        <v>105.444</v>
+        <v>106.02</v>
       </c>
       <c r="E18" s="29" t="n">
         <f aca="false">Baterie!F23</f>
-        <v>123.624</v>
+        <v>123.12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3796,11 +3796,11 @@
       </c>
       <c r="D19" s="24" t="str">
         <f aca="false">TEXT(Baterie!E13,"0")&amp;" ("&amp;TEXT(Baterie!E15,"0")&amp;" – "&amp;TEXT(Baterie!E14,"0")&amp;")"</f>
-        <v>727 (505 – 848)</v>
+        <v>684 (475 – 798)</v>
       </c>
       <c r="E19" s="24" t="str">
         <f aca="false">TEXT(Baterie!F13,"0")&amp;" ("&amp;TEXT(Baterie!F15,"0")&amp;" – "&amp;TEXT(Baterie!F14,"0")&amp;")"</f>
-        <v>727 (505 – 848)</v>
+        <v>684 (475 – 798)</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3813,11 +3813,11 @@
       </c>
       <c r="D20" s="24" t="str">
         <f aca="false">TEXT(Baterie!E31,"0")&amp;" / "&amp;TEXT(Baterie!E32,"0")</f>
-        <v>416 / 660</v>
+        <v>418 / 664</v>
       </c>
       <c r="E20" s="24" t="str">
         <f aca="false">TEXT(Baterie!F31,"0")&amp;" / "&amp;TEXT(Baterie!F32,"0")</f>
-        <v>488 / 774</v>
+        <v>486 / 771</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3849,11 +3849,11 @@
       </c>
       <c r="D22" s="24" t="str">
         <f aca="false">TEXT(Baterie!E18,"0")&amp;" / "&amp;TEXT(Baterie!E19,"0")</f>
-        <v>892 / 1284</v>
+        <v>948 / 1365</v>
       </c>
       <c r="E22" s="24" t="str">
         <f aca="false">TEXT(Baterie!F18,"0")&amp;" / "&amp;TEXT(Baterie!F19,"0")</f>
-        <v>931 / 1341</v>
+        <v>990 / 1426</v>
       </c>
     </row>
   </sheetData>
@@ -4138,7 +4138,7 @@
         <v>135</v>
       </c>
       <c r="C18" s="30" t="n">
-        <v>850</v>
+        <v>800</v>
       </c>
       <c r="D18" s="23" t="s">
         <v>78</v>
@@ -51288,11 +51288,11 @@
       </c>
       <c r="E12" s="38" t="n">
         <f aca="false">ROUNDDOWN(c_U_max/cel_U_max,0)</f>
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="F12" s="38" t="n">
         <f aca="false">ROUNDDOWN(c_U_max/cel_U_max,0)</f>
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="G12" s="33" t="s">
         <v>422</v>
@@ -51311,11 +51311,11 @@
       </c>
       <c r="E13" s="32" t="n">
         <f aca="false">E12*cel_U_nom</f>
-        <v>727.2</v>
+        <v>684</v>
       </c>
       <c r="F13" s="32" t="n">
         <f aca="false">F12*cel_U_nom</f>
-        <v>727.2</v>
+        <v>684</v>
       </c>
       <c r="G13" s="33"/>
     </row>
@@ -51330,11 +51330,11 @@
       </c>
       <c r="E14" s="32" t="n">
         <f aca="false">E12*cel_U_max</f>
-        <v>848.4</v>
+        <v>798</v>
       </c>
       <c r="F14" s="32" t="n">
         <f aca="false">F12*cel_U_max</f>
-        <v>848.4</v>
+        <v>798</v>
       </c>
       <c r="G14" s="33"/>
     </row>
@@ -51349,11 +51349,11 @@
       </c>
       <c r="E15" s="32" t="n">
         <f aca="false">E12*cel_U_min</f>
-        <v>505</v>
+        <v>475</v>
       </c>
       <c r="F15" s="32" t="n">
         <f aca="false">F12*cel_U_min</f>
-        <v>505</v>
+        <v>475</v>
       </c>
       <c r="G15" s="33"/>
     </row>
@@ -51370,11 +51370,11 @@
       </c>
       <c r="E16" s="35" t="n">
         <f aca="false">ROUNDUP(E11/E12,0)</f>
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F16" s="35" t="n">
         <f aca="false">ROUNDUP(F11/F12,0)</f>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G16" s="33"/>
     </row>
@@ -51412,11 +51412,11 @@
       </c>
       <c r="E18" s="32" t="n">
         <f aca="false">E17/E13</f>
-        <v>891.694030514163</v>
+        <v>948.011548230847</v>
       </c>
       <c r="F18" s="32" t="n">
         <f aca="false">F17/F13</f>
-        <v>931.134780144681</v>
+        <v>989.943292574872</v>
       </c>
       <c r="G18" s="33"/>
     </row>
@@ -51433,11 +51433,11 @@
       </c>
       <c r="E19" s="40" t="n">
         <f aca="false">E17/E15</f>
-        <v>1284.03940394039</v>
+        <v>1365.13662945242</v>
       </c>
       <c r="F19" s="40" t="n">
         <f aca="false">F17/F15</f>
-        <v>1340.83408340834</v>
+        <v>1425.51834130782</v>
       </c>
       <c r="G19" s="33" t="s">
         <v>435</v>
@@ -51456,11 +51456,11 @@
       </c>
       <c r="E20" s="35" t="n">
         <f aca="false">ROUNDUP(E19/cel_I,0)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F20" s="35" t="n">
         <f aca="false">ROUNDUP(F19/cel_I,0)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G20" s="33"/>
     </row>
@@ -51477,11 +51477,11 @@
       </c>
       <c r="E21" s="38" t="n">
         <f aca="false">MAX(E16,E20)</f>
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F21" s="38" t="n">
         <f aca="false">MAX(F16,F20)</f>
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G21" s="33"/>
     </row>
@@ -51498,11 +51498,11 @@
       </c>
       <c r="E22" s="38" t="n">
         <f aca="false">E12*E21</f>
-        <v>5858</v>
+        <v>5890</v>
       </c>
       <c r="F22" s="38" t="n">
         <f aca="false">F12*F21</f>
-        <v>6868</v>
+        <v>6840</v>
       </c>
       <c r="G22" s="33"/>
     </row>
@@ -51517,11 +51517,11 @@
       </c>
       <c r="E23" s="41" t="n">
         <f aca="false">E22*E10/3600000</f>
-        <v>105.444</v>
+        <v>106.02</v>
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">F22*F10/3600000</f>
-        <v>123.624</v>
+        <v>123.12</v>
       </c>
       <c r="G23" s="33"/>
     </row>
@@ -51536,11 +51536,11 @@
       </c>
       <c r="E24" s="32" t="n">
         <f aca="false">E21*cel_Cap</f>
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="F24" s="32" t="n">
         <f aca="false">F21*cel_Cap</f>
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="G24" s="33"/>
     </row>
@@ -51555,11 +51555,11 @@
       </c>
       <c r="E25" s="14" t="n">
         <f aca="false">E19/E21</f>
-        <v>44.2772208255308</v>
+        <v>44.0366654662071</v>
       </c>
       <c r="F25" s="14" t="n">
         <f aca="false">F19/F21</f>
-        <v>39.4362965708336</v>
+        <v>39.5977317029949</v>
       </c>
       <c r="G25" s="33" t="s">
         <v>441</v>
@@ -51576,11 +51576,11 @@
       </c>
       <c r="E26" s="14" t="n">
         <f aca="false">E18/E21</f>
-        <v>30.7480700177297</v>
+        <v>30.581017684866</v>
       </c>
       <c r="F26" s="14" t="n">
         <f aca="false">F18/F21</f>
-        <v>27.3863170630789</v>
+        <v>27.4984247937464</v>
       </c>
       <c r="G26" s="33"/>
     </row>
@@ -51618,11 +51618,11 @@
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">E27/c_eta/E13/E21</f>
-        <v>51.6210026175031</v>
+        <v>51.3405489530277</v>
       </c>
       <c r="F28" s="14" t="n">
         <f aca="false">F27/c_eta/F13/F21</f>
-        <v>43.4786125671391</v>
+        <v>43.6565951916829</v>
       </c>
       <c r="G28" s="33"/>
     </row>
@@ -51637,11 +51637,11 @@
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">E27/c_eta/E15/E21</f>
-        <v>74.3342437692045</v>
+        <v>73.9303904923599</v>
       </c>
       <c r="F29" s="14" t="n">
         <f aca="false">F27/c_eta/F15/F21</f>
-        <v>62.6092020966803</v>
+        <v>62.8654970760234</v>
       </c>
       <c r="G29" s="33" t="s">
         <v>446</v>
@@ -51663,11 +51663,11 @@
       </c>
       <c r="E31" s="40" t="n">
         <f aca="false">E22*cel_m</f>
-        <v>415.918</v>
+        <v>418.19</v>
       </c>
       <c r="F31" s="40" t="n">
         <f aca="false">F22*cel_m</f>
-        <v>487.628</v>
+        <v>485.64</v>
       </c>
       <c r="G31" s="33"/>
     </row>
@@ -51682,11 +51682,11 @@
       </c>
       <c r="E32" s="32" t="n">
         <f aca="false">E31/cel_kcp</f>
-        <v>660.187301587302</v>
+        <v>663.793650793651</v>
       </c>
       <c r="F32" s="32" t="n">
         <f aca="false">F31/cel_kcp</f>
-        <v>774.012698412698</v>
+        <v>770.857142857143</v>
       </c>
       <c r="G32" s="33" t="s">
         <v>450</v>
@@ -51722,11 +51722,11 @@
       </c>
       <c r="E34" s="32" t="n">
         <f aca="false">E31/E8*100</f>
-        <v>17.655064097122</v>
+        <v>17.7515069190933</v>
       </c>
       <c r="F34" s="32" t="n">
         <f aca="false">F31/F8*100</f>
-        <v>19.8222764227642</v>
+        <v>19.7414634146341</v>
       </c>
       <c r="G34" s="33"/>
     </row>
@@ -51741,11 +51741,11 @@
       </c>
       <c r="E35" s="32" t="n">
         <f aca="false">E32/E8*100</f>
-        <v>28.023911265273</v>
+        <v>28.1769951096719</v>
       </c>
       <c r="F35" s="32" t="n">
         <f aca="false">F32/F8*100</f>
-        <v>31.4639308297845</v>
+        <v>31.335656213705</v>
       </c>
       <c r="G35" s="33"/>
     </row>

</xml_diff>